<commit_message>
feat(metas): M1.1-1.4 a 8000, M9 a 5000; meta disponibilidad a 90%
Metas mensuales (vigentes desde julio 2026):
- Millalemu 1.1/1.2/1.3/1.4: 7000 -> 8000 m3
- Millalemu 9: 7000 -> 5000 m3
Actualizadas en el Excel maestro (hoja CONFIGURACIÓN, E24-E27, E30),
en METAS_DEFAULT (GENERAR_HTML) y en METAS (generar_snapshots).
Los meses ya cerrados conservan sus metas (meta.json de su snapshot).

Disponibilidad mecánica: umbral 'bajo meta' 80% -> 90% en el semáforo,
alertas y coloreado por equipo (nivel crítico <60% sin cambios).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dashboard_CosechaForestal.xlsx
+++ b/Dashboard_CosechaForestal.xlsx
@@ -17286,7 +17286,7 @@
         </is>
       </c>
       <c r="E24" s="106" t="n">
-        <v>7000</v>
+        <v>8000</v>
       </c>
       <c r="F24" s="107">
         <f>IF(CONFIGURACIÓN!$C$10=0,0,ROUND(E24/CONFIGURACIÓN!$C$10,1))</f>
@@ -17319,7 +17319,7 @@
         </is>
       </c>
       <c r="E25" s="106" t="n">
-        <v>7000</v>
+        <v>8000</v>
       </c>
       <c r="F25" s="107">
         <f>IF(CONFIGURACIÓN!$C$10=0,0,ROUND(E25/CONFIGURACIÓN!$C$10,1))</f>
@@ -17352,7 +17352,7 @@
         </is>
       </c>
       <c r="E26" s="106" t="n">
-        <v>7000</v>
+        <v>8000</v>
       </c>
       <c r="F26" s="107">
         <f>IF(CONFIGURACIÓN!$C$10=0,0,ROUND(E26/CONFIGURACIÓN!$C$10,1))</f>
@@ -17385,7 +17385,7 @@
         </is>
       </c>
       <c r="E27" s="106" t="n">
-        <v>7000</v>
+        <v>8000</v>
       </c>
       <c r="F27" s="107">
         <f>IF(CONFIGURACIÓN!$C$10=0,0,ROUND(E27/CONFIGURACIÓN!$C$10,1))</f>
@@ -17484,7 +17484,7 @@
         </is>
       </c>
       <c r="E30" s="106" t="n">
-        <v>7000</v>
+        <v>5000</v>
       </c>
       <c r="F30" s="107">
         <f>IF(CONFIGURACIÓN!$C$10=0,0,ROUND(E30/CONFIGURACIÓN!$C$10,1))</f>

</xml_diff>

<commit_message>
feat(metas): M1.1-1.4 a 8000, M9 a 5000; meta disponibilidad a 90% (#3)
Metas mensuales (vigentes desde julio 2026):
- Millalemu 1.1/1.2/1.3/1.4: 7000 -> 8000 m3
- Millalemu 9: 7000 -> 5000 m3
Actualizadas en el Excel maestro (hoja CONFIGURACIÓN, E24-E27, E30),
en METAS_DEFAULT (GENERAR_HTML) y en METAS (generar_snapshots).
Los meses ya cerrados conservan sus metas (meta.json de su snapshot).

Disponibilidad mecánica: umbral 'bajo meta' 80% -> 90% en el semáforo,
alertas y coloreado por equipo (nivel crítico <60% sin cambios).

Co-authored-by: cesarg-lab <cesgoinos@gmail.com>
Co-authored-by: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dashboard_CosechaForestal.xlsx
+++ b/Dashboard_CosechaForestal.xlsx
@@ -17286,7 +17286,7 @@
         </is>
       </c>
       <c r="E24" s="106" t="n">
-        <v>7000</v>
+        <v>8000</v>
       </c>
       <c r="F24" s="107">
         <f>IF(CONFIGURACIÓN!$C$10=0,0,ROUND(E24/CONFIGURACIÓN!$C$10,1))</f>
@@ -17319,7 +17319,7 @@
         </is>
       </c>
       <c r="E25" s="106" t="n">
-        <v>7000</v>
+        <v>8000</v>
       </c>
       <c r="F25" s="107">
         <f>IF(CONFIGURACIÓN!$C$10=0,0,ROUND(E25/CONFIGURACIÓN!$C$10,1))</f>
@@ -17352,7 +17352,7 @@
         </is>
       </c>
       <c r="E26" s="106" t="n">
-        <v>7000</v>
+        <v>8000</v>
       </c>
       <c r="F26" s="107">
         <f>IF(CONFIGURACIÓN!$C$10=0,0,ROUND(E26/CONFIGURACIÓN!$C$10,1))</f>
@@ -17385,7 +17385,7 @@
         </is>
       </c>
       <c r="E27" s="106" t="n">
-        <v>7000</v>
+        <v>8000</v>
       </c>
       <c r="F27" s="107">
         <f>IF(CONFIGURACIÓN!$C$10=0,0,ROUND(E27/CONFIGURACIÓN!$C$10,1))</f>
@@ -17484,7 +17484,7 @@
         </is>
       </c>
       <c r="E30" s="106" t="n">
-        <v>7000</v>
+        <v>5000</v>
       </c>
       <c r="F30" s="107">
         <f>IF(CONFIGURACIÓN!$C$10=0,0,ROUND(E30/CONFIGURACIÓN!$C$10,1))</f>

</xml_diff>

<commit_message>
Metas Julio 2026: M7 7000→8060, M9 5000→5940; umbral disponibilidad verde 90%→92%
M5 se mantiene en 7000. Cambios en Excel CONFIGURACIÓN (E29/E30),
METAS_DEFAULT/METAS de fallback y coloreo de disponibilidad.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dashboard_CosechaForestal.xlsx
+++ b/Dashboard_CosechaForestal.xlsx
@@ -17451,7 +17451,7 @@
         </is>
       </c>
       <c r="E29" s="106" t="n">
-        <v>7000</v>
+        <v>8060</v>
       </c>
       <c r="F29" s="107">
         <f>IF(CONFIGURACIÓN!$C$10=0,0,ROUND(E29/CONFIGURACIÓN!$C$10,1))</f>
@@ -17484,7 +17484,7 @@
         </is>
       </c>
       <c r="E30" s="106" t="n">
-        <v>5000</v>
+        <v>5940</v>
       </c>
       <c r="F30" s="107">
         <f>IF(CONFIGURACIÓN!$C$10=0,0,ROUND(E30/CONFIGURACIÓN!$C$10,1))</f>

</xml_diff>

<commit_message>
Meta M9: 5.940 -> 10.000 m3 (total mes 59.000 -> 63.060)
Excel CONFIGURACION fila 30 por cirugia XML (graficos intactos):
E30=10000, I30=10501 (volteo, +3x167), J30=10334 (madereo, +2x167), K30=10000.
Defaults sincronizados en GENERAR_HTML, compute_kpis, generar_snapshots
y generar_tablero_faena.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dashboard_CosechaForestal.xlsx
+++ b/Dashboard_CosechaForestal.xlsx
@@ -17556,7 +17556,7 @@
         </is>
       </c>
       <c r="E30" s="106" t="n">
-        <v>5940</v>
+        <v>10000</v>
       </c>
       <c r="F30" s="107">
         <f>IF(CONFIGURACIÓN!$C$10=0,0,ROUND(E30/CONFIGURACIÓN!$C$10,1))</f>
@@ -17572,13 +17572,13 @@
         </is>
       </c>
       <c r="I30" s="106" t="n">
-        <v>6441</v>
+        <v>10501</v>
       </c>
       <c r="J30" s="106" t="n">
-        <v>6274</v>
+        <v>10334</v>
       </c>
       <c r="K30" s="106" t="n">
-        <v>5940</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="31" ht="19.5" customHeight="1" s="150">

</xml_diff>

<commit_message>
M9: colchon de volteo/madereo con el ritmo real (313 m3/dia)
Las columnas I/J venian del p90 de julio (167 m3/dia), cuando la faena
trozaba 105-147/dia. Desde el 07-08 M9 corre 232-342/dia (media 272,
p90 313), que es el ritmo que el propio informe muestra. Con eso:
  volteo  I30 = 10.000 + 3x313 = 10.939  (antes 10.501)
  madereo J30 = 10.000 + 2x313 = 10.626  (antes 10.334)
E30/K30 siguen en 10.000. Ahora el objetivo de buffer de la hoja 1 y el
saldo de la hoja 2 hablan del mismo ritmo.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dashboard_CosechaForestal.xlsx
+++ b/Dashboard_CosechaForestal.xlsx
@@ -17572,10 +17572,10 @@
         </is>
       </c>
       <c r="I30" s="106" t="n">
-        <v>10501</v>
+        <v>10939</v>
       </c>
       <c r="J30" s="106" t="n">
-        <v>10334</v>
+        <v>10626</v>
       </c>
       <c r="K30" s="106" t="n">
         <v>10000</v>

</xml_diff>